<commit_message>
master_control: закупка 0am325025ae 900 → 700
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Btw2doetXoQivbsfVavokQ
</commit_message>
<xml_diff>
--- a/data/master_control.xlsx
+++ b/data/master_control.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Товары" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Нераспознанные фото" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Товары" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нераспознанные фото" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -171,13 +171,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -196,13 +199,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -221,13 +227,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -246,13 +255,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -271,13 +283,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -296,13 +311,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -321,13 +339,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -346,13 +367,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -371,13 +395,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -396,13 +423,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -421,13 +451,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -446,13 +479,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -471,13 +507,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -496,13 +535,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -521,13 +563,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -546,13 +591,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -571,13 +619,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -596,13 +647,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -621,13 +675,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -646,13 +703,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId20"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -671,13 +731,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId21"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -696,13 +759,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId22"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -721,13 +787,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId23"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -746,13 +815,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId24"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -771,13 +843,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId25"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -796,13 +871,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId26"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -821,13 +899,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId27"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -846,13 +927,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId28"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -871,13 +955,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId29"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -896,13 +983,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId30"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -921,13 +1011,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId31"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -946,13 +1039,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId32"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -971,13 +1067,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId33"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -996,13 +1095,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId34"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId34"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1021,13 +1123,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId35"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId35"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1046,13 +1151,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId36"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1071,13 +1179,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId37"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1096,13 +1207,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId38"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1121,13 +1235,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId39"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1146,13 +1263,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId40"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1171,13 +1291,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId41"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1196,13 +1319,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId42"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1221,13 +1347,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId43"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1246,13 +1375,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId44"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1271,13 +1403,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId45"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1296,13 +1431,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId46"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId46"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1321,13 +1459,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId47"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId47"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1346,13 +1487,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId48"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId48"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1371,13 +1515,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId49"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId49"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1396,13 +1543,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId50"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId50"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1421,13 +1571,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId51"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId51"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1446,13 +1599,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId52"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId52"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1471,13 +1627,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId53"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId53"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1496,13 +1655,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId54"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId54"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1521,13 +1683,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId55"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId55"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1546,13 +1711,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId56"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId56"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1571,13 +1739,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId57"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId57"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1596,13 +1767,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId58"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId58"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1621,13 +1795,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId59"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId59"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1646,13 +1823,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId60"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId60"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1671,13 +1851,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId61"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId61"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1696,13 +1879,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId62"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId62"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1721,13 +1907,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId63"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId63"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1746,13 +1935,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId64"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId64"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1771,13 +1963,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId65"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId65"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1796,13 +1991,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId66"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId66"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1821,13 +2019,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId67"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId67"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1846,13 +2047,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId68"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId68"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1871,13 +2075,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId69"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId69"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1896,13 +2103,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId70"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId70"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1921,13 +2131,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId71"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId71"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1946,13 +2159,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId72"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId72"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1971,13 +2187,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId73"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId73"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1996,13 +2215,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId74"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId74"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2021,13 +2243,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId75"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId75"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2046,13 +2271,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId76"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId76"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2071,13 +2299,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId77"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId77"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2096,13 +2327,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId78"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId78"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2121,13 +2355,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId79"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId79"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2146,13 +2383,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId80"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId80"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2171,13 +2411,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId81"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId81"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2196,13 +2439,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId82"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId82"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2221,13 +2467,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId83"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId83"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2246,13 +2495,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId84"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId84"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2271,13 +2523,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId85"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId85"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2296,13 +2551,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId86"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId86"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2321,13 +2579,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId87"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId87"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2346,13 +2607,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId88"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId88"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2371,13 +2635,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId89"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId89"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2396,13 +2663,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId90"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId90"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2421,13 +2691,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId91"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId91"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2446,13 +2719,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId92"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId92"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2471,13 +2747,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId93"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId93"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2496,13 +2775,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId94"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId94"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2521,13 +2803,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId95"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId95"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2546,13 +2831,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId96"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId96"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2571,13 +2859,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId97"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId97"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2596,13 +2887,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId98"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId98"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2621,13 +2915,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId99"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId99"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2646,13 +2943,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId100"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId100"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2671,13 +2971,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId101"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId101"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2696,13 +2999,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId102"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId102"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2721,13 +3027,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId103"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId103"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2746,13 +3055,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId104"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId104"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2771,13 +3083,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId105"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId105"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2796,13 +3111,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId106"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId106"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2821,13 +3139,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId107"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId107"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2846,13 +3167,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId108"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId108"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2871,13 +3195,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId109"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId109"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2896,13 +3223,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId110"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId110"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2921,13 +3251,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId111"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId111"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2946,13 +3279,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId112"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId112"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2971,13 +3307,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId113"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId113"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2996,13 +3335,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId114"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId114"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3021,13 +3363,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId115"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId115"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3046,13 +3391,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId116"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId116"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3071,13 +3419,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId117"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId117"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3096,13 +3447,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId118"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId118"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3121,13 +3475,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId119"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId119"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6183,7 +6540,7 @@
       <c r="Y35" s="2" t="n"/>
       <c r="Z35" s="2" t="n"/>
       <c r="AA35" s="2" t="n">
-        <v>900</v>
+        <v>700</v>
       </c>
       <c r="AB35" s="2" t="n"/>
     </row>

</xml_diff>

<commit_message>
Цены Ozon/WB (одобрено владельцем): 0am325091f 2850->3350, 0am325025D 2850->3350, 0am325025u 4350->5350
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Btw2dpuabcabgcDaPC8mav
</commit_message>
<xml_diff>
--- a/data/master_control.xlsx
+++ b/data/master_control.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Товары" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Нераспознанные фото" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Товары" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нераспознанные фото" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -171,13 +171,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -196,13 +199,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -221,13 +227,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -246,13 +255,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -271,13 +283,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -296,13 +311,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -321,13 +339,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -346,13 +367,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -371,13 +395,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -396,13 +423,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -421,13 +451,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -446,13 +479,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -471,13 +507,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -496,13 +535,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -521,13 +563,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -546,13 +591,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -571,13 +619,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -596,13 +647,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -621,13 +675,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -646,13 +703,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId20"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -671,13 +731,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId21"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -696,13 +759,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId22"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -721,13 +787,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId23"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -746,13 +815,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId24"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -771,13 +843,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId25"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -796,13 +871,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId26"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -821,13 +899,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId27"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -846,13 +927,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId28"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -871,13 +955,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId29"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -896,13 +983,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId30"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -921,13 +1011,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId31"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -946,13 +1039,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId32"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -971,13 +1067,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId33"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -996,13 +1095,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId34"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId34"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1021,13 +1123,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId35"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId35"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1046,13 +1151,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId36"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1071,13 +1179,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId37"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1096,13 +1207,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId38"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1121,13 +1235,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId39"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1146,13 +1263,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId40"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1171,13 +1291,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId41"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1196,13 +1319,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId42"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1221,13 +1347,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId43"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1246,13 +1375,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId44"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1271,13 +1403,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId45"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1296,13 +1431,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId46"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId46"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1321,13 +1459,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId47"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId47"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1346,13 +1487,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId48"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId48"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1371,13 +1515,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId49"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId49"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1396,13 +1543,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId50"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId50"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1421,13 +1571,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId51"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId51"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1446,13 +1599,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId52"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId52"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1471,13 +1627,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId53"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId53"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1496,13 +1655,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId54"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId54"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1521,13 +1683,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId55"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId55"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1546,13 +1711,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId56"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId56"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1571,13 +1739,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId57"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId57"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1596,13 +1767,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId58"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId58"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1621,13 +1795,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId59"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId59"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1646,13 +1823,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId60"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId60"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1671,13 +1851,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId61"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId61"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1696,13 +1879,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId62"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId62"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1721,13 +1907,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId63"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId63"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1746,13 +1935,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId64"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId64"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1771,13 +1963,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId65"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId65"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1796,13 +1991,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId66"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId66"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1821,13 +2019,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId67"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId67"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1846,13 +2047,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId68"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId68"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1871,13 +2075,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId69"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId69"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1896,13 +2103,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId70"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId70"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1921,13 +2131,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId71"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId71"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1946,13 +2159,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId72"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId72"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1971,13 +2187,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId73"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId73"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1996,13 +2215,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId74"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId74"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2021,13 +2243,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId75"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId75"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2046,13 +2271,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId76"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId76"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2071,13 +2299,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId77"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId77"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2096,13 +2327,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId78"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId78"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2121,13 +2355,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId79"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId79"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2146,13 +2383,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId80"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId80"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2171,13 +2411,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId81"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId81"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2196,13 +2439,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId82"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId82"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2221,13 +2467,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId83"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId83"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2246,13 +2495,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId84"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId84"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2271,13 +2523,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId85"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId85"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2296,13 +2551,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId86"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId86"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2321,13 +2579,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId87"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId87"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2346,13 +2607,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId88"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId88"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2371,13 +2635,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId89"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId89"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2396,13 +2663,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId90"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId90"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2421,13 +2691,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId91"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId91"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2446,13 +2719,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId92"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId92"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2471,13 +2747,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId93"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId93"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2496,13 +2775,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId94"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId94"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2521,13 +2803,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId95"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId95"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2546,13 +2831,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId96"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId96"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2571,13 +2859,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId97"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId97"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2596,13 +2887,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId98"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId98"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2621,13 +2915,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId99"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId99"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2646,13 +2943,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId100"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId100"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2671,13 +2971,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId101"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId101"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2696,13 +2999,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId102"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId102"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2721,13 +3027,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId103"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId103"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2746,13 +3055,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId104"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId104"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2771,13 +3083,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId105"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId105"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2796,13 +3111,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId106"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId106"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2821,13 +3139,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId107"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId107"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2846,13 +3167,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId108"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId108"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2871,13 +3195,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId109"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId109"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2896,13 +3223,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId110"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId110"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2921,13 +3251,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId111"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId111"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2946,13 +3279,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId112"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId112"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2971,13 +3307,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId113"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId113"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2996,13 +3335,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId114"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId114"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3021,13 +3363,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId115"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId115"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3046,13 +3391,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId116"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId116"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3071,13 +3419,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId117"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId117"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3096,13 +3447,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId118"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId118"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3121,13 +3475,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId119"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId119"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5681,7 +6038,7 @@
         </is>
       </c>
       <c r="H29" s="2" t="n">
-        <v>2850</v>
+        <v>3350</v>
       </c>
       <c r="I29" s="2" t="n">
         <v>5000</v>
@@ -5690,7 +6047,7 @@
         <v>151</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>2850</v>
+        <v>3350</v>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
@@ -6850,7 +7207,7 @@
         </is>
       </c>
       <c r="H44" s="2" t="n">
-        <v>4350</v>
+        <v>5350</v>
       </c>
       <c r="I44" s="2" t="n">
         <v>6000</v>
@@ -6859,7 +7216,7 @@
         <v>151</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>4350</v>
+        <v>5350</v>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
@@ -7642,7 +7999,7 @@
         </is>
       </c>
       <c r="H54" s="2" t="n">
-        <v>2850</v>
+        <v>3350</v>
       </c>
       <c r="I54" s="2" t="n">
         <v>5000</v>
@@ -7651,7 +8008,7 @@
         <v>191</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>2850</v>
+        <v>3350</v>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Ozon «нет» для 4 дублей (plita-filtr, plita-filtr-pylniki-sal-orig, remkomplekt-shtokov-orig, -v2) — согласовано владельцем
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Btw2dnNbUBQBzqB24HwuZ7
</commit_message>
<xml_diff>
--- a/data/master_control.xlsx
+++ b/data/master_control.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Товары" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Нераспознанные фото" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Товары" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нераспознанные фото" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -171,13 +171,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -196,13 +199,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -221,13 +227,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -246,13 +255,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -271,13 +283,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -296,13 +311,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -321,13 +339,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -346,13 +367,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -371,13 +395,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -396,13 +423,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -421,13 +451,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -446,13 +479,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -471,13 +507,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -496,13 +535,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -521,13 +563,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -546,13 +591,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -571,13 +619,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -596,13 +647,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -621,13 +675,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -646,13 +703,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId20"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -671,13 +731,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId21"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -696,13 +759,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId22"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -721,13 +787,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId23"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -746,13 +815,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId24"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -771,13 +843,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId25"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -796,13 +871,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId26"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -821,13 +899,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId27"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -846,13 +927,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId28"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -871,13 +955,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId29"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -896,13 +983,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId30"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -921,13 +1011,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId31"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -946,13 +1039,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId32"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -971,13 +1067,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId33"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -996,13 +1095,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId34"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId34"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1021,13 +1123,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId35"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId35"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1046,13 +1151,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId36"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1071,13 +1179,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId37"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1096,13 +1207,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId38"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1121,13 +1235,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId39"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1146,13 +1263,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId40"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1171,13 +1291,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId41"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1196,13 +1319,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId42"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1221,13 +1347,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId43"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1246,13 +1375,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId44"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1271,13 +1403,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId45"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1296,13 +1431,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId46"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId46"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1321,13 +1459,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId47"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId47"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1346,13 +1487,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId48"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId48"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1371,13 +1515,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId49"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId49"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1396,13 +1543,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId50"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId50"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1421,13 +1571,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId51"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId51"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1446,13 +1599,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId52"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId52"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1471,13 +1627,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId53"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId53"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1496,13 +1655,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId54"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId54"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1521,13 +1683,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId55"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId55"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1546,13 +1711,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId56"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId56"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1571,13 +1739,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId57"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId57"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1596,13 +1767,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId58"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId58"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1621,13 +1795,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId59"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId59"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1646,13 +1823,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId60"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId60"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1671,13 +1851,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId61"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId61"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1696,13 +1879,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId62"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId62"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1721,13 +1907,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId63"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId63"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1746,13 +1935,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId64"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId64"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1771,13 +1963,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId65"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId65"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1796,13 +1991,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId66"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId66"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1821,13 +2019,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId67"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId67"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1846,13 +2047,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId68"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId68"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1871,13 +2075,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId69"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId69"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1896,13 +2103,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId70"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId70"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1921,13 +2131,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId71"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId71"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1946,13 +2159,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId72"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId72"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1971,13 +2187,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId73"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId73"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1996,13 +2215,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId74"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId74"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2021,13 +2243,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId75"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId75"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2046,13 +2271,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId76"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId76"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2071,13 +2299,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId77"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId77"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2096,13 +2327,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId78"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId78"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2121,13 +2355,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId79"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId79"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2146,13 +2383,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId80"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId80"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2171,13 +2411,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId81"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId81"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2196,13 +2439,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId82"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId82"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2221,13 +2467,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId83"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId83"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2246,13 +2495,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId84"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId84"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2271,13 +2523,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId85"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId85"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2296,13 +2551,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId86"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId86"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2321,13 +2579,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId87"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId87"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2346,13 +2607,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId88"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId88"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2371,13 +2635,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId89"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId89"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2396,13 +2663,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId90"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId90"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2421,13 +2691,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId91"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId91"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2446,13 +2719,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId92"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId92"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2471,13 +2747,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId93"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId93"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2496,13 +2775,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId94"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId94"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2521,13 +2803,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId95"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId95"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2546,13 +2831,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId96"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId96"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2571,13 +2859,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId97"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId97"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2596,13 +2887,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId98"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId98"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2621,13 +2915,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId99"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId99"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2646,13 +2943,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId100"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId100"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2671,13 +2971,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId101"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId101"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2696,13 +2999,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId102"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId102"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2721,13 +3027,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId103"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId103"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2746,13 +3055,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId104"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId104"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2771,13 +3083,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId105"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId105"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2796,13 +3111,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId106"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId106"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2821,13 +3139,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId107"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId107"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2846,13 +3167,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId108"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId108"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2871,13 +3195,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId109"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId109"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2896,13 +3223,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId110"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId110"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2921,13 +3251,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId111"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId111"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2946,13 +3279,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId112"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId112"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2971,13 +3307,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId113"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId113"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2996,13 +3335,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId114"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId114"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3021,13 +3363,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId115"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId115"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3046,13 +3391,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId116"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId116"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3071,13 +3419,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId117"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId117"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3096,13 +3447,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId118"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId118"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3121,13 +3475,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId119"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId119"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3146,13 +3503,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId120"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId120"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10957,7 +11317,7 @@
       <c r="M96" s="2" t="inlineStr"/>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>Ozon: нет (дубль SPU / не создаём)</t>
+          <t>Ozon: нет (дубль SPU / не создаём); 27.10.2026: Ozon «нет» — дубль существующей карточки (SPU)</t>
         </is>
       </c>
       <c r="O96" s="2" t="inlineStr">
@@ -10972,7 +11332,7 @@
       </c>
       <c r="Q96" s="2" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>нет</t>
         </is>
       </c>
       <c r="R96" s="2" t="n"/>
@@ -11347,7 +11707,7 @@
       </c>
       <c r="N101" s="2" t="inlineStr">
         <is>
-          <t>Ozon: нет (дубль SPU / не создаём)</t>
+          <t>Ozon: нет (дубль SPU / не создаём); 27.10.2026: Ozon «нет» — дубль существующей карточки (SPU)</t>
         </is>
       </c>
       <c r="O101" s="2" t="inlineStr">
@@ -11362,7 +11722,7 @@
       </c>
       <c r="Q101" s="2" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>нет</t>
         </is>
       </c>
       <c r="R101" s="2" t="n"/>
@@ -12511,7 +12871,7 @@
       <c r="M116" s="2" t="inlineStr"/>
       <c r="N116" s="2" t="inlineStr">
         <is>
-          <t>Ozon: нет (дубль SPU / не создаём)</t>
+          <t>Ozon: нет (дубль SPU / не создаём); 27.10.2026: Ozon «нет» — дубль существующей карточки (SPU)</t>
         </is>
       </c>
       <c r="O116" s="2" t="inlineStr">
@@ -12526,7 +12886,7 @@
       </c>
       <c r="Q116" s="2" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>нет</t>
         </is>
       </c>
       <c r="R116" s="2" t="n"/>
@@ -12585,7 +12945,11 @@
         </is>
       </c>
       <c r="M117" s="2" t="inlineStr"/>
-      <c r="N117" s="2" t="inlineStr"/>
+      <c r="N117" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026: Ozon «нет» — дубль существующей карточки (SPU)</t>
+        </is>
+      </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
           <t>remkomplekt-shtokov-orig-v2_1.png</t>
@@ -12596,7 +12960,11 @@
           <t>8708409909</t>
         </is>
       </c>
-      <c r="Q117" s="2" t="n"/>
+      <c r="Q117" s="2" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
       <c r="R117" s="2" t="n"/>
       <c r="S117" s="2" t="n"/>
       <c r="T117" s="2" t="n"/>

</xml_diff>